<commit_message>
Getting more experience in using python libraries.
</commit_message>
<xml_diff>
--- a/exam.xlsx
+++ b/exam.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kibo Underwood</t>
+          <t>Velma Clemons</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -475,27 +475,27 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A+</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Giselle Lancaster</t>
+          <t>Kirsten Mcdowell</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -509,27 +509,27 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="G3" t="n">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Zenaida Decker</t>
+          <t>Kibo Underwood</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -543,27 +543,27 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="G4" t="n">
-        <v>55.00000000000001</v>
+        <v>81</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Velma Clemons</t>
+          <t>Giselle Lancaster</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -577,27 +577,27 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="E5" t="n">
         <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="G5" t="n">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gillian Tillman</t>
+          <t>Louis Mcgee</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -611,27 +611,27 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="G6" t="n">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Phyllis Paul</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -645,27 +645,27 @@
         </is>
       </c>
       <c r="D7" t="n">
+        <v>69</v>
+      </c>
+      <c r="E7" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" t="n">
         <v>31</v>
       </c>
-      <c r="E7" t="n">
-        <v>100</v>
-      </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>69</v>
       </c>
-      <c r="G7" t="n">
-        <v>31</v>
-      </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Phyllis Paul</t>
+          <t>Zenaida Decker</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -679,20 +679,20 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="E8" t="n">
         <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="G8" t="n">
-        <v>18</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
     </row>
@@ -713,27 +713,27 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E9" t="n">
         <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="G9" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kirsten Mcdowell</t>
+          <t>Gillian Tillman</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -747,16 +747,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="E10" t="n">
         <v>100</v>
       </c>
       <c r="F10" t="n">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="G10" t="n">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -767,7 +767,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Louis Mcgee</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -781,16 +781,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="E11" t="n">
         <v>100</v>
       </c>
       <c r="F11" t="n">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="G11" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>

</xml_diff>